<commit_message>
Upload folder for excel gone
</commit_message>
<xml_diff>
--- a/uploads/IS1.xlsx
+++ b/uploads/IS1.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{415C0021-8B0B-4111-8043-241DA7149283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1215BB3D-5FB5-4D73-8839-4DCF8CD492AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Income statement" sheetId="2" r:id="rId1"/>
@@ -1028,7 +1028,7 @@
       <c r="D3" s="12"/>
       <c r="E3" s="21"/>
       <c r="F3" s="41">
-        <v>45517</v>
+        <v>45882</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="44"/>
@@ -1901,15 +1901,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="26" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ac37c1753acd5e330d2062ccec26ea66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b340c7101c92c5120abd06486f94548" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -2209,6 +2200,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B25903B0-7748-4EC8-9AE6-30C7129DC7C9}">
   <ds:schemaRefs>
@@ -2229,14 +2229,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{078BDA64-E289-47E3-BE11-83ECE4B2E315}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40E5EBD5-9A8B-4FB3-9210-57091BDE8FDC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2257,6 +2249,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{078BDA64-E289-47E3-BE11-83ECE4B2E315}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata"/>
 </file>
</xml_diff>